<commit_message>
Refresh the P6 demo: glass look-ahead with a WBS tree, and the new Repair XER fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -1622,7 +1622,7 @@
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="I23" s="5" t="n"/>
@@ -3660,7 +3660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3723,31 +3723,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Logic vs reality</t>
+          <t>Logic quality</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F2" t="n">
-        <v>49.15</v>
+        <v>8.33</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>29 finish-to-start links were violated in execution: the successor started before the predecessor finished.</t>
+          <t>5 activities have a start or finish that nothing controls, even though they do have relationships.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Either the logic is wrong and should be changed to SS with a lag, or the work genuinely happened out of order and the sequence needs re-planning. Left alone, the remaining schedule is driven by logic the team is already ignoring.</t>
+          <t>An activity whose successors are all SS can slip its finish forever without moving anything downstream. Add the missing FS/FF link so both ends of the activity are tied into the network.</t>
         </is>
       </c>
     </row>
@@ -3759,31 +3759,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Logic quality</t>
+          <t>Logic vs reality</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Out-of-sequence progress</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F3" t="n">
-        <v>8.33</v>
+        <v>6.78</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>5 activities have a start or finish that nothing controls, even though they do have relationships.</t>
+          <t>4 open activities have progressed against logic that is still waiting on its predecessor.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>An activity whose successors are all SS can slip its finish forever without moving anything downstream. Add the missing FS/FF link so both ends of the activity are tied into the network.</t>
+          <t>P6 holds their remaining work behind a link the site has already ignored, so the forecast is wrong. Change each link to the relationships the work actually followed - Repair XER does this - or re-plan the sequence.</t>
         </is>
       </c>
     </row>
@@ -3856,6 +3856,42 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>This work is invisible to earned value and to any resource histogram, so forecasts understate what is left to do. Load them, or exclude them from the EVM basis deliberately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>As-built record</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>29</v>
+      </c>
+      <c r="E6" t="n">
+        <v>59</v>
+      </c>
+      <c r="F6" t="n">
+        <v>49.15</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>29 relationships were broken by work that has since caught up - the successor started or finished before the logic allowed.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>These no longer move any date, so they do not affect the forecast. They matter for as-built and delay analysis, where the logic should describe how the work was really done. Repair XER can re-type them to the relationships the actual dates satisfy.</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3921,27 +3957,23 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A1250</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Build package 25</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>A1240</t>
-        </is>
-      </c>
+          <t>Build package 32</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>started 35d before its predecessor finished</t>
+          <t>finish drives nothing (SS successors only)</t>
         </is>
       </c>
     </row>
@@ -3953,27 +3985,23 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A1290</t>
+          <t>A1390</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Build package 29</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>A1280</t>
-        </is>
-      </c>
+          <t>Build package 39</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>started 11d before its predecessor finished</t>
+          <t>start is not driven by any predecessor (FF/SF only)</t>
         </is>
       </c>
     </row>
@@ -3985,27 +4013,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A1050</t>
+          <t>A1430</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Design package 05</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>A1040</t>
-        </is>
-      </c>
+          <t>Build package 43</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>finish drives nothing (SS successors only)</t>
         </is>
       </c>
     </row>
@@ -4017,27 +4041,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A1120</t>
+          <t>A1520</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Design package 12</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>A1110</t>
-        </is>
-      </c>
+          <t>Build package 52</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>start is not driven by any predecessor (FF/SF only)</t>
         </is>
       </c>
     </row>
@@ -4049,27 +4069,23 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Dangling logic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1540</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Design package 17</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>A1160</t>
-        </is>
-      </c>
+          <t>Build package 54</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>finish drives nothing (SS successors only)</t>
         </is>
       </c>
     </row>
@@ -4086,22 +4102,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1180</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Design package 18</t>
+          <t>Build package 35</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started before its predecessor finished (predecessor still open)</t>
         </is>
       </c>
     </row>
@@ -4118,22 +4134,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A1360</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Build package 21</t>
+          <t>Build package 36</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>A1200</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started before its predecessor finished (predecessor still open)</t>
         </is>
       </c>
     </row>
@@ -4150,22 +4166,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A1230</t>
+          <t>A1370</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Build package 23</t>
+          <t>Build package 37</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>A1220</t>
+          <t>A1360</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started before its predecessor finished (predecessor still open)</t>
         </is>
       </c>
     </row>
@@ -4182,22 +4198,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Build package 31</t>
+          <t>Build package 38</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>A1300</t>
+          <t>A1370</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started before its predecessor finished (predecessor still open)</t>
         </is>
       </c>
     </row>
@@ -4209,887 +4225,1035 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>High float caused by missing successors</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A1020</t>
+          <t>A1590</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Design package 02</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>A1010</t>
-        </is>
-      </c>
+          <t>Build package 59</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>started 6d before its predecessor finished</t>
+          <t>50d float and no successor</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Remaining work with no resources or cost</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A1070</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Design package 07</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>A1060</t>
-        </is>
-      </c>
+          <t>Build package 38</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>started 6d before its predecessor finished</t>
+          <t>no resource or cost assigned</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Remaining work with no resources or cost</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A1240</t>
+          <t>A1450</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Build package 24</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>A1230</t>
-        </is>
-      </c>
+          <t>Build package 45</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>started 6d before its predecessor finished</t>
+          <t>no resource or cost assigned</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Remaining work with no resources or cost</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A1010</t>
+          <t>A1520</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Design package 01</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>A1000</t>
-        </is>
-      </c>
+          <t>Build package 52</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>no resource or cost assigned</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A1040</t>
+          <t>A1250</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Design package 04</t>
+          <t>Build package 25</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1240</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 35d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A1150</t>
+          <t>A1290</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Design package 15</t>
+          <t>Build package 29</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>A1140</t>
+          <t>A1280</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 11d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A1200</t>
+          <t>A1050</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Build package 20</t>
+          <t>Design package 05</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A1190</t>
+          <t>A1040</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A1270</t>
+          <t>A1120</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Build package 27</t>
+          <t>Design package 12</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A1260</t>
+          <t>A1110</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A1320</t>
+          <t>A1170</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Build package 32</t>
+          <t>Design package 17</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1160</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A1160</t>
+          <t>A1180</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Design package 16</t>
+          <t>Design package 18</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>A1150</t>
+          <t>A1170</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>started 2d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A1280</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Build package 28</t>
+          <t>Build package 21</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A1270</t>
+          <t>A1200</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>started 2d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1230</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Design package 03</t>
+          <t>Build package 23</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>A1020</t>
+          <t>A1220</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A1060</t>
+          <t>A1310</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Design package 06</t>
+          <t>Build package 31</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>A1050</t>
+          <t>A1300</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A1080</t>
+          <t>A1020</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Design package 08</t>
+          <t>Design package 02</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>A1070</t>
+          <t>A1010</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 6d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A1090</t>
+          <t>A1070</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Design package 09</t>
+          <t>Design package 07</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A1080</t>
+          <t>A1060</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 6d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A1100</t>
+          <t>A1240</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Design package 10</t>
+          <t>Build package 24</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>A1090</t>
+          <t>A1230</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 6d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A1140</t>
+          <t>A1010</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Design package 14</t>
+          <t>Design package 01</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>A1130</t>
+          <t>A1000</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>A1190</t>
+          <t>A1040</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Design package 19</t>
+          <t>Design package 04</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A1180</t>
+          <t>A1030</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A1300</t>
+          <t>A1150</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Build package 30</t>
+          <t>Design package 15</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A1290</t>
+          <t>A1140</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Out-of-sequence progress</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>A1340</t>
+          <t>A1200</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Build package 34</t>
+          <t>Build package 20</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>A1330</t>
+          <t>A1190</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A1320</t>
+          <t>A1270</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Build package 32</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>Build package 27</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>A1260</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>A1390</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Build package 39</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>Build package 32</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>A1310</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>start is not driven by any predecessor (FF/SF only)</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A1430</t>
+          <t>A1160</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Build package 43</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>Design package 16</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>A1150</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>started 2d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A1520</t>
+          <t>A1280</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Build package 52</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+          <t>Build package 28</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>A1270</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>start is not driven by any predecessor (FF/SF only)</t>
+          <t>started 2d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Dangling logic</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A1540</t>
+          <t>A1030</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Build package 54</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+          <t>Design package 03</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>A1020</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>started 1d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>High float caused by missing successors</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>A1590</t>
+          <t>A1060</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Build package 59</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr"/>
+          <t>Design package 06</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>A1050</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>50d float and no successor</t>
+          <t>started 1d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Remaining work with no resources or cost</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A1380</t>
+          <t>A1080</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Build package 38</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>Design package 08</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>A1070</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>started 1d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Remaining work with no resources or cost</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>A1450</t>
+          <t>A1090</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Build package 45</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr"/>
+          <t>Design package 09</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>A1080</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>started 1d before its predecessor finished</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Remaining work with no resources or cost</t>
+          <t>Work recorded out of sequence</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>A1520</t>
+          <t>A1100</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Build package 52</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr"/>
+          <t>Design package 10</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>A1090</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>A1140</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Design package 14</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>A1130</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>A1190</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Design package 19</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>A1180</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A1300</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Build package 30</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>A1290</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>A1340</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Build package 34</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>A1330</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -14171,7 +14335,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-22T20:17:10Z</t>
+          <t>2026-09-23T19:21:52Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the P6 demo: redesigned Schedule Health, counted the DCMA way
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -5345,19 +5345,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>≤ 5% of activities</t>
+          <t>≤ 5% of incomplete activities</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.0% (0 of 60)</t>
+          <t>0.0% (0 of 27)</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -5385,14 +5385,14 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0 of 59 relationships</t>
+          <t>0 of 27 relationships into incomplete work</t>
         </is>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -5405,7 +5405,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Excessive lags</t>
+          <t>Lags</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
@@ -5415,22 +5415,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>≤ 5% with lag &gt; 5d</t>
+          <t>≤ 5% of relationships into incomplete work with any positive lag</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5.08% (3 of 59)</t>
+          <t>14.81% (4 of 27)</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="H4" t="n">
-        <v>5.08</v>
+        <v>14.81</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -5455,19 +5455,23 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>84.75% FS (50 of 59)</t>
+          <t>85.19% FS (23 of 27)</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="H5" t="n">
-        <v>84.75</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
+        <v>85.19</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Counted on 27 relationships into incomplete work, as DCMA does; links into finished work no longer drive anything.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -5485,26 +5489,26 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>≤ 5% of activities</t>
+          <t>≤ 5% of incomplete activities</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3.33% (2 of 60)</t>
+          <t>3.7% (1 of 27)</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="H6" t="n">
-        <v>3.33</v>
+        <v>3.7</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1 additional soft constraints present (not counted).</t>
+          <t>Counts the DCMA list: Mandatory Start/Finish, Start/Finish On and Start/Finish On or Before. 0 other constraints present (not counted).</t>
         </is>
       </c>
     </row>
@@ -5634,19 +5638,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3 of 60</t>
+          <t>3 of 27</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>3</v>
       </c>
       <c r="G10" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="H10" t="n">
-        <v>5</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+        <v>11.11</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Forecast dates are P6's early dates from the last reschedule. If they are in the past, the file was not rescheduled after statusing - press F9 in P6 and export again.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -5669,17 +5677,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13.79% (8 of 58)</t>
+          <t>11.54% (3 of 26)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G11" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="H11" t="n">
-        <v>13.79</v>
+        <v>11.54</v>
       </c>
       <c r="I11" t="inlineStr"/>
     </row>
@@ -5716,7 +5724,11 @@
       <c r="H12" t="n">
         <v>8.33</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Measured against P6's planned dates (the target dates in the export), the usual stand-in when the file does not carry its baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -5786,7 +5798,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Critical path length 161 working days; project total float -3 days.</t>
+          <t>Critical path length 161 working days; total float -3 days (lowest float of any open activity - the file's stored dates were not produced by a reschedule, so the finishing activity's stored float cannot be relied on).</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5837,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>33 completed vs 36 planned complete. Start execution index 1.000 (39 of 39 started).</t>
+          <t>33 completed vs 36 planned complete. Start execution index 1.000 (39 of 39 started). Measured against P6's planned dates.</t>
         </is>
       </c>
     </row>
@@ -5840,7 +5852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5895,24 +5907,24 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Excessive lags</t>
+          <t>Lags</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Design package 17</t>
+          <t>Build package 34</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>lag 10.0d exceeds 5d</t>
+          <t>lag 10.0d</t>
         </is>
       </c>
     </row>
@@ -5922,24 +5934,24 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Excessive lags</t>
+          <t>Lags</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A1340</t>
+          <t>A1440</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Build package 34</t>
+          <t>Build package 44</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>lag 10.0d exceeds 5d</t>
+          <t>lag 2.0d</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5961,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Excessive lags</t>
+          <t>Lags</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -5966,24 +5978,36 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>lag 10.0d exceeds 5d</t>
+          <t>lag 10.0d</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Relationship types</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+          <t>Lags</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A1550</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Build package 55</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>lag 2.0d</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -6017,36 +6041,18 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hard constraints</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>A1120</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Design package 12</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>hard constraint</t>
-        </is>
-      </c>
+          <t>Relationship types</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -6059,17 +6065,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A1330</t>
+          <t>A1440</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Build package 33</t>
+          <t>Build package 44</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -6620,17 +6626,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Design package 03</t>
+          <t>Build package 38</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -6653,21 +6659,21 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A1100</t>
+          <t>A1450</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Design package 10</t>
+          <t>Build package 45</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -6686,21 +6692,21 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1520</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Design package 17</t>
+          <t>Build package 52</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -6710,87 +6716,87 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Resources / cost loading</t>
+          <t>Missed activities</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A1240</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Build package 24</t>
+          <t>Build package 32</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>planned to finish before data date, still open</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Resources / cost loading</t>
+          <t>Missed activities</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Build package 31</t>
+          <t>Build package 34</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>planned to finish before data date, still open</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Resources / cost loading</t>
+          <t>Missed activities</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A1380</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Build package 38</t>
+          <t>Build package 35</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -6803,93 +6809,89 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>planned to finish before data date, still open</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Resources / cost loading</t>
+          <t>Critical path test</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>A1450</t>
+          <t>A1390</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Build package 45</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
+          <t>Build package 39</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>test activity</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Resources / cost loading</t>
+          <t>Baseline Execution Index (BEI)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A1520</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Build package 52</t>
+          <t>Build package 32</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>planned to be complete, not finished</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Missed activities</t>
+          <t>Baseline Execution Index (BEI)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A1320</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Build package 32</t>
+          <t>Build package 34</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -6902,27 +6904,27 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>planned to finish before data date, still open</t>
+          <t>planned to be complete, not finished</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Missed activities</t>
+          <t>Baseline Execution Index (BEI)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A1340</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Build package 34</t>
+          <t>Build package 35</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -6934,167 +6936,6 @@
         <v>0</v>
       </c>
       <c r="G35" t="inlineStr">
-        <is>
-          <t>planned to finish before data date, still open</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>11</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Missed activities</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>A1350</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Build package 35</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>planned to finish before data date, still open</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>12</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Critical path test</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>A1390</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Build package 39</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>test activity</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>14</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Baseline Execution Index (BEI)</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>A1320</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Build package 32</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>planned to be complete, not finished</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>14</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Baseline Execution Index (BEI)</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>A1340</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Build package 34</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>planned to be complete, not finished</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>14</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Baseline Execution Index (BEI)</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>A1350</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Build package 35</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" t="inlineStr">
         <is>
           <t>planned to be complete, not finished</t>
         </is>
@@ -14335,7 +14176,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23T19:21:52Z</t>
+          <t>2026-09-24T18:13:16Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the P6 demo: redesigned, verified Insights
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -1622,7 +1622,7 @@
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="I23" s="5" t="n"/>
@@ -1652,7 +1652,7 @@
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>3 critical or high</t>
+          <t>4 critical or high</t>
         </is>
       </c>
       <c r="I24" s="5" t="n"/>
@@ -3660,17 +3660,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="78" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="78" customWidth="1" min="8" max="8"/>
+    <col width="90" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3696,20 +3697,25 @@
       </c>
       <c r="E1" s="13" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Out of</t>
         </is>
       </c>
       <c r="F1" s="13" t="inlineStr">
         <is>
+          <t>Counted against</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
           <t>%</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>What it means</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
@@ -3735,17 +3741,22 @@
         <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
-      </c>
-      <c r="F2" t="n">
-        <v>8.33</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>5 activities have a start or finish that nothing controls, even though they do have relationships.</t>
-        </is>
+        <v>26</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>open activities</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>19.23</v>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>5 open activities have a start or finish that nothing controls, even though they do have relationships.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>An activity whose successors are all SS can slip its finish forever without moving anything downstream. Add the missing FS/FF link so both ends of the activity are tied into the network.</t>
         </is>
@@ -3771,17 +3782,22 @@
         <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>59</v>
-      </c>
-      <c r="F3" t="n">
-        <v>6.78</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>4 open activities have progressed against logic that is still waiting on its predecessor.</t>
-        </is>
+        <v>27</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>relationships into open work</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>14.81</v>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>4 relationships into open work were broken by progress: 4 activities have progressed against logic that is still waiting on its predecessor.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>P6 holds their remaining work behind a link the site has already ignored, so the forecast is wrong. Change each link to the relationships the work actually followed - Repair XER does this - or re-plan the sequence.</t>
         </is>
@@ -3795,101 +3811,157 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Progress integrity</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Running well over their planned duration</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>in-progress activities</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2 in-progress activities have been open for at least half as long again as planned (and ten working days more).</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>These are the classic signature of work that stopped but was never suspended, or of activities scoped too coarsely. Confirm which are genuinely active, suspend the rest, and give the live ones a realistic remaining duration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Logic quality</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>High float caused by missing successors</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D5" t="n">
         <v>1</v>
       </c>
-      <c r="E4" t="n">
-        <v>60</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.67</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>1 activities combine float above 44 days with no successor at all.</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="E5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>open activities</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1 open activity combines float above 44 days with no successor at all.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>This float is an artefact of missing logic, not real slack - the activity simply floats to the end of the project. Add the successor that reflects what the work actually enables.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Resources</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Remaining work with no resources or cost</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>60</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>3 incomplete activities carry neither resources nor cost.</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>This work is invisible to earned value and to any resource histogram, so forecasts understate what is left to do. Load them, or exclude them from the EVM basis deliberately.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Resources</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Remaining work with no resources or cost</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>open work activities</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>3 open activities carry neither resources nor cost, in a programme where 86% of the work is loaded.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>This work is invisible to earned value and to any resource histogram, so forecasts understate what is left to do. Load them, or exclude them from the EVM basis deliberately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>As-built record</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Work recorded out of sequence</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>29</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E7" t="n">
         <v>59</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>relationships</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
         <v>49.15</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>29 relationships were broken by work that has since caught up - the successor started or finished before the logic allowed.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>These no longer move any date, so they do not affect the forecast. They matter for as-built and delay analysis, where the logic should describe how the work was really done. Repair XER can re-type them to the relationships the actual dates satisfy.</t>
         </is>
@@ -3906,7 +3978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3973,7 +4045,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>finish drives nothing (SS/SF successors only)</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4101,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>finish drives nothing (SS/SF successors only)</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4157,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>finish drives nothing (SS successors only)</t>
+          <t>finish drives nothing (SS/SF successors only)</t>
         </is>
       </c>
     </row>
@@ -4225,79 +4297,79 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>High float caused by missing successors</t>
+          <t>Running well over their planned duration</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A1590</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Build package 59</t>
+          <t>Build package 32</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>50d float and no successor</t>
+          <t>open 19 working days against 5 planned, at 80%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Remaining work with no resources or cost</t>
+          <t>Running well over their planned duration</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A1380</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Build package 38</t>
+          <t>Build package 34</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>open 15 working days against 3 planned, at 40%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Remaining work with no resources or cost</t>
+          <t>High float caused by missing successors</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A1450</t>
+          <t>A1590</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Build package 45</t>
+          <t>Build package 59</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>no resource or cost assigned</t>
+          <t>50d float and no successor</t>
         </is>
       </c>
     </row>
@@ -4314,12 +4386,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A1520</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Build package 52</t>
+          <t>Build package 38</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -4332,64 +4404,56 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Work recorded out of sequence</t>
+          <t>Remaining work with no resources or cost</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A1250</t>
+          <t>A1450</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Build package 25</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>A1240</t>
-        </is>
-      </c>
+          <t>Build package 45</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>started 35d before its predecessor finished</t>
+          <t>no resource or cost assigned</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Work recorded out of sequence</t>
+          <t>Remaining work with no resources or cost</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A1290</t>
+          <t>A1520</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Build package 29</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>A1280</t>
-        </is>
-      </c>
+          <t>Build package 52</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>started 11d before its predecessor finished</t>
+          <t>no resource or cost assigned</t>
         </is>
       </c>
     </row>
@@ -4406,22 +4470,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A1050</t>
+          <t>A1250</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Design package 05</t>
+          <t>Build package 25</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>A1040</t>
+          <t>A1240</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started 35d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4438,22 +4502,22 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A1120</t>
+          <t>A1290</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Design package 12</t>
+          <t>Build package 29</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>A1110</t>
+          <t>A1280</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>started 7d before its predecessor finished</t>
+          <t>started 11d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4470,17 +4534,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1050</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Design package 17</t>
+          <t>Design package 05</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A1160</t>
+          <t>A1040</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -4502,17 +4566,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A1180</t>
+          <t>A1120</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Design package 18</t>
+          <t>Design package 12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1110</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4534,17 +4598,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A1210</t>
+          <t>A1170</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Build package 21</t>
+          <t>Design package 17</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A1200</t>
+          <t>A1160</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4566,17 +4630,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A1230</t>
+          <t>A1180</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Build package 23</t>
+          <t>Design package 18</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>A1220</t>
+          <t>A1170</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4598,17 +4662,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1210</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Build package 31</t>
+          <t>Build package 21</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>A1300</t>
+          <t>A1200</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4630,22 +4694,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A1020</t>
+          <t>A1230</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Design package 02</t>
+          <t>Build package 23</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>A1010</t>
+          <t>A1220</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>started 6d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4662,22 +4726,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A1070</t>
+          <t>A1310</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Design package 07</t>
+          <t>Build package 31</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A1060</t>
+          <t>A1300</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>started 6d before its predecessor finished</t>
+          <t>started 7d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4694,17 +4758,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A1240</t>
+          <t>A1020</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Build package 24</t>
+          <t>Design package 02</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>A1230</t>
+          <t>A1010</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -4726,22 +4790,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A1010</t>
+          <t>A1070</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Design package 01</t>
+          <t>Design package 07</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>A1000</t>
+          <t>A1060</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 6d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4758,22 +4822,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>A1040</t>
+          <t>A1240</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Design package 04</t>
+          <t>Build package 24</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1230</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>started 4d before its predecessor finished</t>
+          <t>started 6d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4790,17 +4854,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A1150</t>
+          <t>A1010</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Design package 15</t>
+          <t>Design package 01</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A1140</t>
+          <t>A1000</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -4822,17 +4886,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>A1200</t>
+          <t>A1040</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Build package 20</t>
+          <t>Design package 04</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>A1190</t>
+          <t>A1030</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -4854,17 +4918,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A1270</t>
+          <t>A1150</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Build package 27</t>
+          <t>Design package 15</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>A1260</t>
+          <t>A1140</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -4886,17 +4950,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>A1320</t>
+          <t>A1200</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Build package 32</t>
+          <t>Build package 20</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1190</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -4918,22 +4982,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A1160</t>
+          <t>A1270</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Design package 16</t>
+          <t>Build package 27</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A1150</t>
+          <t>A1260</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>started 2d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4950,22 +5014,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A1280</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Build package 28</t>
+          <t>Build package 32</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>A1270</t>
+          <t>A1310</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>started 2d before its predecessor finished</t>
+          <t>started 4d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -4982,22 +5046,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1160</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Design package 03</t>
+          <t>Design package 16</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>A1020</t>
+          <t>A1150</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 2d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -5014,22 +5078,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>A1060</t>
+          <t>A1280</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Design package 06</t>
+          <t>Build package 28</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>A1050</t>
+          <t>A1270</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>started 1d before its predecessor finished</t>
+          <t>started 2d before its predecessor finished</t>
         </is>
       </c>
     </row>
@@ -5046,17 +5110,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>A1080</t>
+          <t>A1030</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Design package 08</t>
+          <t>Design package 03</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>A1070</t>
+          <t>A1020</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -5078,17 +5142,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>A1090</t>
+          <t>A1060</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Design package 09</t>
+          <t>Design package 06</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>A1080</t>
+          <t>A1050</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -5110,17 +5174,17 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>A1100</t>
+          <t>A1080</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Design package 10</t>
+          <t>Design package 08</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>A1090</t>
+          <t>A1070</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -5142,17 +5206,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>A1140</t>
+          <t>A1090</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Design package 14</t>
+          <t>Design package 09</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>A1130</t>
+          <t>A1080</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -5174,17 +5238,17 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A1190</t>
+          <t>A1100</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Design package 19</t>
+          <t>Design package 10</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>A1180</t>
+          <t>A1090</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -5206,17 +5270,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A1300</t>
+          <t>A1140</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Build package 30</t>
+          <t>Design package 14</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>A1290</t>
+          <t>A1130</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -5238,20 +5302,84 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
+          <t>A1190</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Design package 19</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>A1180</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>A1300</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Build package 30</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>A1290</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>started 1d before its predecessor finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Work recorded out of sequence</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
           <t>A1340</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Build package 34</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>A1330</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>started 1d before its predecessor finished</t>
         </is>
@@ -14176,7 +14304,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-27T17:20:03Z</t>
+          <t>2026-09-27T18:32:50Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the P6 demo: Risk Analysis in working days, glass design
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -14277,7 +14277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -14304,7 +14304,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-27T18:57:13Z</t>
+          <t>2026-09-27T19:04:06Z</t>
         </is>
       </c>
     </row>
@@ -14401,42 +14401,62 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Buffer to P80 (days)</t>
+          <t>P80 after the planned finish (working days)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>64</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Target date</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2025-07-31</t>
-        </is>
+          <t>P80 after the planned finish (calendar days)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Confidence in target %</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>28.5</v>
+          <t>Target date</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>P80 vs target (days)</t>
+          <t>Confidence in target %</t>
         </is>
       </c>
       <c r="B15" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P80 vs target (working days)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>P80 vs target (calendar days)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>29</v>
       </c>
     </row>
@@ -14694,7 +14714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14702,9 +14722,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="33" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14735,17 +14756,22 @@
       </c>
       <c r="F1" s="13" t="inlineStr">
         <is>
-          <t>Mean impact (working d)</t>
+          <t>Mean impact (working days)</t>
         </is>
       </c>
       <c r="G1" s="13" t="inlineStr">
         <is>
-          <t>Finish delay when it occurs (d)</t>
+          <t>Finish delay when it occurs (working days)</t>
         </is>
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
-          <t>Expected delay (d)</t>
+          <t>Expected delay (working days)</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>Expected delay (calendar days)</t>
         </is>
       </c>
     </row>
@@ -14775,9 +14801,12 @@
         <v>13.6</v>
       </c>
       <c r="G2" t="n">
-        <v>20.3</v>
+        <v>14.5</v>
       </c>
       <c r="H2" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="I2" t="n">
         <v>6.9</v>
       </c>
     </row>
@@ -14807,9 +14836,12 @@
         <v>7.1</v>
       </c>
       <c r="G3" t="n">
-        <v>11.1</v>
+        <v>7.9</v>
       </c>
       <c r="H3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -14839,9 +14871,12 @@
         <v>10.2</v>
       </c>
       <c r="G4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="I4" t="n">
         <v>4.3</v>
       </c>
     </row>
@@ -14865,7 +14900,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="29" customWidth="1" min="10" max="10"/>
@@ -14905,7 +14940,7 @@
       </c>
       <c r="G1" s="13" t="inlineStr">
         <is>
-          <t>P80 vs plan (d)</t>
+          <t>P80 vs plan (working days)</t>
         </is>
       </c>
       <c r="H1" s="13" t="inlineStr">
@@ -14961,7 +14996,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="H2" t="n">
         <v>0.2</v>

</xml_diff>

<commit_message>
Refresh the P6 demo: NEC4 and Activities reviewed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -1532,7 +1532,7 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="11" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L18" s="5" t="n"/>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2025-06-26</t>
+          <t>2025-02-12</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1819,7 +1819,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>45.5</v>
+        <v>37.5</v>
       </c>
     </row>
   </sheetData>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Planned Completion is 2025-06-26. No Completion Date has been entered, so terminal float cannot be assessed.</t>
+          <t>Planned Completion is 2025-02-12. No Completion Date has been entered, so terminal float cannot be assessed.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0 of 60 activities (0.0%) have a missing predecessor or successor, so their timing is not driven by the programme logic.</t>
+          <t>0 of 27 remaining activities (0.0%) have a missing predecessor or successor, so their timing is not driven by the programme logic.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -2080,9 +2080,9 @@
           <t>Order and timing of the work of the Client and Others</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>No activities appear to represent work by the Client or Others.</t>
+          <t>No activity names identify work by the Client or Others - confirm whether it is shown under other wording.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2150,9 +2150,9 @@
           <t>Provisions for time risk allowances</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>No activities are identifiable as time risk allowances.</t>
+          <t>No activity is named as a time risk allowance - check whether the allowances are shown under other wording or buried in durations.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2290,9 +2290,9 @@
           <t>Dates needed — information from Others</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2302,16 +2302,16 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>20 activities reference information from Others.</t>
+          <t>No activities clearly reference information from Others.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Confirm each carries the date it is needed by, so late information can be evidenced.</t>
+          <t>If information from Others is required, show it on the programme with the date needed, so late information can be evidenced. If genuinely not required, no action.</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2 hard constraints override the logic; 29 finish-to-start links were violated in execution.</t>
+          <t>0 hard constraints on remaining work override the logic; 4 links into open work are broken by out-of-sequence progress.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -2500,9 +2500,9 @@
           <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2512,12 +2512,16 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>No evidence the programme contradicts its own data date.</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
+          <t>The programme was not rescheduled after it was last changed: 17 links into work not yet started are broken by its own stored dates (by up to 25 working days); 3 unfinished activities are still forecast to finish before the data date.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Reschedule (F9) against the data date before submitting. A programme showing dates its own logic no longer produces does not represent the Contractor's plans and is an easy ground for non-acceptance.</t>
+        </is>
+      </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
@@ -2772,7 +2776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2822,12 +2826,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A1250</t>
+          <t>A1370</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Build package 25</t>
+          <t>Build package 37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
@@ -2845,12 +2849,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A1300</t>
+          <t>A1400</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Build package 30</t>
+          <t>Build package 40</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -2868,12 +2872,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A1310</t>
+          <t>A1430</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Build package 31</t>
+          <t>Build package 43</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -2891,12 +2895,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A1370</t>
+          <t>A1460</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Build package 37</t>
+          <t>Build package 46</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -2914,12 +2918,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A1400</t>
+          <t>A1530</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Build package 40</t>
+          <t>Build package 53</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -2932,17 +2936,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Provisions for float</t>
+          <t>Statement of how the work is done — resources</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A1430</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Build package 43</t>
+          <t>Build package 38</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -2955,17 +2959,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Provisions for float</t>
+          <t>Statement of how the work is done — resources</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A1460</t>
+          <t>A1450</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Build package 46</t>
+          <t>Build package 45</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -2978,17 +2982,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Provisions for float</t>
+          <t>Statement of how the work is done — resources</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A1530</t>
+          <t>A1520</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Build package 53</t>
+          <t>Build package 52</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -2996,531 +3000,623 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Plans shown are practicable</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A1000</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Design package 00</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+          <t>Build package 35</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>progressed before A1340 (FS)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Plans shown are practicable</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A1010</t>
+          <t>A1360</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Design package 01</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>Build package 36</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>progressed before A1350 (FS)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Plans shown are practicable</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A1020</t>
+          <t>A1370</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Design package 02</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Build package 37</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>progressed before A1360 (FS)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Plans shown are practicable</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A1030</t>
+          <t>A1380</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Design package 03</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+          <t>Build package 38</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>progressed before A1370 (FS)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A1040</t>
+          <t>A1400</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Design package 04</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Build package 40</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>starts before A1390 allows, by 25 working days</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A1050</t>
+          <t>A1540</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Design package 05</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+          <t>Build package 54</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>starts before A1530 allows, by 25 working days</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>A1060</t>
+          <t>A1590</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Design package 06</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>Build package 59</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>starts before A1580 allows, by 25 working days</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A1070</t>
+          <t>A1510</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Design package 07</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Build package 51</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>starts before A1500 allows, by 12 working days</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A1080</t>
+          <t>A1460</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Design package 08</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>Build package 46</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>starts before A1450 allows, by 8 working days</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>A1090</t>
+          <t>A1420</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Design package 09</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>Build package 42</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>starts before A1410 allows, by 7 working days</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A1100</t>
+          <t>A1490</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Design package 10</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>Build package 49</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>starts before A1480 allows, by 5 working days</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A1110</t>
+          <t>A1570</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Design package 11</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Build package 57</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>starts before A1560 allows, by 5 working days</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A1120</t>
+          <t>A1410</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Design package 12</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>Build package 41</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>starts before A1400 allows, by 4 working days</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>A1130</t>
+          <t>A1500</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Design package 13</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr"/>
+          <t>Build package 50</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>starts before A1490 allows, by 4 working days</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A1140</t>
+          <t>A1530</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Design package 14</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>Build package 53</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>starts before A1520 allows, by 4 working days</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>A1150</t>
+          <t>A1560</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Design package 15</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+          <t>Build package 56</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>starts before A1550 allows, by 4 working days</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>A1160</t>
+          <t>A1450</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Design package 16</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>Build package 45</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>starts before A1440 allows, by 2 working days</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A1170</t>
+          <t>A1470</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Design package 17</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
+          <t>Build package 47</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>starts before A1460 allows, by 2 working days</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>A1180</t>
+          <t>A1480</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Design package 18</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>Build package 48</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>starts before A1470 allows, by 2 working days</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dates needed — information from Others</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A1190</t>
+          <t>A1430</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Design package 19</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
+          <t>Build package 43</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>starts before A1420 allows, by 1 working days</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Statement of how the work is done — resources</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>A1380</t>
+          <t>A1580</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Build package 38</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr"/>
+          <t>Build package 58</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>starts before A1570 allows, by 1 working days</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Statement of how the work is done — resources</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>A1450</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Build package 45</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr"/>
+          <t>Build package 32</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>unfinished, forecast before the data date</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>31.2</t>
+          <t>31.3</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Statement of how the work is done — resources</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>A1520</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Build package 52</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
+          <t>Build package 34</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>unfinished, forecast before the data date</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3530,43 +3626,51 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Plans shown are practicable</t>
+          <t>Represents the Contractor's plans realistically</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A1120</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Design package 12</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr"/>
+          <t>Build package 35</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>unfinished, forecast before the data date</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>31.3</t>
+          <t>32.1</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Plans shown are practicable</t>
+          <t>Effect of progress on the timing of remaining work</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>A1330</t>
+          <t>A1320</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Build package 33</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr"/>
+          <t>Build package 32</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>incomplete but forecast in the past</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3581,12 +3685,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>A1320</t>
+          <t>A1340</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Build package 32</t>
+          <t>Build package 34</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3608,42 +3712,15 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>A1340</t>
+          <t>A1350</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Build package 34</t>
+          <t>Build package 35</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
-        <is>
-          <t>incomplete but forecast in the past</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>32.1</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Effect of progress on the timing of remaining work</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>A1350</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Build package 35</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
         <is>
           <t>incomplete but forecast in the past</t>
         </is>
@@ -7166,10 +7243,10 @@
         <v>22236</v>
       </c>
       <c r="H2" t="n">
-        <v>10700</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>11536</v>
+        <v>22236</v>
       </c>
     </row>
     <row r="3">
@@ -7197,10 +7274,10 @@
         <v>44400</v>
       </c>
       <c r="H3" t="n">
-        <v>13440</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>30960</v>
+        <v>44400</v>
       </c>
     </row>
     <row r="4">
@@ -7228,10 +7305,10 @@
         <v>68334.55</v>
       </c>
       <c r="H4" t="n">
-        <v>28440</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>39894.55</v>
+        <v>68334.55</v>
       </c>
     </row>
     <row r="5">
@@ -7259,10 +7336,10 @@
         <v>71920</v>
       </c>
       <c r="H5" t="n">
-        <v>28440</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>43480</v>
+        <v>71920</v>
       </c>
     </row>
     <row r="6">
@@ -7290,10 +7367,10 @@
         <v>93435</v>
       </c>
       <c r="H6" t="n">
-        <v>36760</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>56675</v>
+        <v>93435</v>
       </c>
     </row>
     <row r="7">
@@ -7321,10 +7398,10 @@
         <v>106908</v>
       </c>
       <c r="H7" t="n">
-        <v>52640</v>
+        <v>13680</v>
       </c>
       <c r="I7" t="n">
-        <v>63080</v>
+        <v>102040</v>
       </c>
     </row>
     <row r="8">
@@ -7340,10 +7417,10 @@
         <v>127116.08</v>
       </c>
       <c r="H8" t="n">
-        <v>61836.08</v>
+        <v>22876.08</v>
       </c>
       <c r="I8" t="n">
-        <v>65280</v>
+        <v>104240</v>
       </c>
     </row>
     <row r="9">
@@ -7359,10 +7436,10 @@
         <v>154548.77</v>
       </c>
       <c r="H9" t="n">
-        <v>88388.77</v>
+        <v>49428.77</v>
       </c>
       <c r="I9" t="n">
-        <v>66160</v>
+        <v>105120</v>
       </c>
     </row>
     <row r="10">
@@ -7378,10 +7455,10 @@
         <v>179000</v>
       </c>
       <c r="H10" t="n">
-        <v>109040</v>
+        <v>70080</v>
       </c>
       <c r="I10" t="n">
-        <v>69960</v>
+        <v>108920</v>
       </c>
     </row>
     <row r="11">
@@ -7397,10 +7474,10 @@
         <v>198721.57</v>
       </c>
       <c r="H11" t="n">
-        <v>125161.57</v>
+        <v>86201.57000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>73560</v>
+        <v>112520</v>
       </c>
     </row>
     <row r="12">
@@ -7416,10 +7493,10 @@
         <v>227495.9</v>
       </c>
       <c r="H12" t="n">
-        <v>141688.63</v>
+        <v>102728.63</v>
       </c>
       <c r="I12" t="n">
-        <v>85807.27</v>
+        <v>124767.27</v>
       </c>
     </row>
     <row r="13">
@@ -7435,10 +7512,10 @@
         <v>253200</v>
       </c>
       <c r="H13" t="n">
-        <v>152120</v>
+        <v>113160</v>
       </c>
       <c r="I13" t="n">
-        <v>101080</v>
+        <v>140040</v>
       </c>
     </row>
     <row r="14">
@@ -7454,10 +7531,10 @@
         <v>266400</v>
       </c>
       <c r="H14" t="n">
-        <v>152120</v>
+        <v>113160</v>
       </c>
       <c r="I14" t="n">
-        <v>114280</v>
+        <v>153240</v>
       </c>
     </row>
     <row r="15">
@@ -7473,10 +7550,10 @@
         <v>269400</v>
       </c>
       <c r="H15" t="n">
-        <v>152120</v>
+        <v>113160</v>
       </c>
       <c r="I15" t="n">
-        <v>117280</v>
+        <v>156240</v>
       </c>
     </row>
   </sheetData>
@@ -7912,7 +7989,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -14304,7 +14381,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-27T19:04:06Z</t>
+          <t>2026-09-27T21:59:27Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the P6 demo: Health checked against P6's Check Schedule, Apply progress tested in P6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -5713,7 +5713,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Counts the DCMA list: Mandatory Start/Finish, Start/Finish On and Start/Finish On or Before. 0 other constraints present (not counted).</t>
+          <t>Counts the DCMA list: Mandatory Start/Finish, Start/Finish On and Start/Finish On or Before. 0 other constraints in force (not counted; start constraints on work already started are spent).</t>
         </is>
       </c>
     </row>
@@ -5808,17 +5808,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>11.11% (3 of 27)</t>
+          <t>11.54% (3 of 26)</t>
         </is>
       </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
       <c r="G9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H9" t="n">
-        <v>11.11</v>
+        <v>11.54</v>
       </c>
       <c r="I9" t="inlineStr"/>
     </row>
@@ -14381,7 +14381,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-04T22:22:05Z</t>
+          <t>2026-10-21T17:04:05Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh the P6 demo: Health against a baseline, with P6's late activities
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/demo-data/sample-export.xlsx
+++ b/demo/demo-data/sample-export.xlsx
@@ -5473,7 +5473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5931,7 +5931,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Measured against P6's planned dates (the target dates in the export), the usual stand-in when the file does not carry its baseline.</t>
+          <t>Measured against P6's planned dates (the target dates in the export). Once P6 reschedules, the planned dates of work not yet started follow its forecast, so load a baseline in Baseline &amp; Delay to measure against it.</t>
         </is>
       </c>
     </row>
@@ -6042,7 +6042,46 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>33 completed vs 36 planned complete. Start execution index 1.000 (39 of 39 started). Measured against P6's planned dates.</t>
+          <t>33 completed vs 36 planned complete. Start execution index 1.000 (39 of 39 started). Measured against P6's planned dates, which for work not yet started follow the forecast once P6 reschedules - load a baseline in Baseline &amp; Delay.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Late activities (as P6 reports it; not scored)</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>≤ 5% of incomplete activities</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.0% (0 of 26)</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>26</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No baseline is loaded, so this compares with P6's planned dates, which follow the forecast for work not yet started - load a baseline in Baseline &amp; Delay.</t>
         </is>
       </c>
     </row>
@@ -14381,7 +14420,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-21T17:04:05Z</t>
+          <t>2026-10-21T17:51:42Z</t>
         </is>
       </c>
     </row>

</xml_diff>